<commit_message>
cambio calculo de tiempo de computo
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_NEH(InsertionFirstImprovement).xlsx
+++ b/code/resultados/NWJSSP_OADG_NEH(InsertionFirstImprovement).xlsx
@@ -15,6 +15,7 @@
     <sheet name="ft20r" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="tai_j10_m10_1" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="tai_j10_m10_1r" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="tai_j100_m10_1" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +429,7 @@
         <v>314</v>
       </c>
       <c r="B1" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2">
@@ -512,7 +513,7 @@
         <v>9808</v>
       </c>
       <c r="B1" t="n">
-        <v>113</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2">
@@ -566,7 +567,7 @@
         <v>10077</v>
       </c>
       <c r="B1" t="n">
-        <v>54</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2">
@@ -620,7 +621,7 @@
         <v>17291</v>
       </c>
       <c r="B1" t="n">
-        <v>1393</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="2">
@@ -704,7 +705,7 @@
         <v>18991</v>
       </c>
       <c r="B1" t="n">
-        <v>710</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="2">
@@ -788,7 +789,7 @@
         <v>97668</v>
       </c>
       <c r="B1" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
@@ -842,7 +843,7 @@
         <v>96328</v>
       </c>
       <c r="B1" t="n">
-        <v>88</v>
+        <v>131</v>
       </c>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>
@@ -888,4 +889,328 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:CV2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>6477982</v>
+      </c>
+      <c r="B1" t="n">
+        <v>3600039</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>52418</v>
+      </c>
+      <c r="B2" t="n">
+        <v>87942</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38566</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22837</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100969</v>
+      </c>
+      <c r="F2" t="n">
+        <v>8179</v>
+      </c>
+      <c r="G2" t="n">
+        <v>49044</v>
+      </c>
+      <c r="H2" t="n">
+        <v>120158</v>
+      </c>
+      <c r="I2" t="n">
+        <v>126086</v>
+      </c>
+      <c r="J2" t="n">
+        <v>27671</v>
+      </c>
+      <c r="K2" t="n">
+        <v>8072</v>
+      </c>
+      <c r="L2" t="n">
+        <v>170</v>
+      </c>
+      <c r="M2" t="n">
+        <v>84385</v>
+      </c>
+      <c r="N2" t="n">
+        <v>26866</v>
+      </c>
+      <c r="O2" t="n">
+        <v>67576</v>
+      </c>
+      <c r="P2" t="n">
+        <v>14199</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>94241</v>
+      </c>
+      <c r="R2" t="n">
+        <v>6480</v>
+      </c>
+      <c r="S2" t="n">
+        <v>51127</v>
+      </c>
+      <c r="T2" t="n">
+        <v>34664</v>
+      </c>
+      <c r="U2" t="n">
+        <v>94163</v>
+      </c>
+      <c r="V2" t="n">
+        <v>91022</v>
+      </c>
+      <c r="W2" t="n">
+        <v>89653</v>
+      </c>
+      <c r="X2" t="n">
+        <v>121999</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>108928</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>77518</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>30594</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>64756</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>14154</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>981</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>5454</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>68265</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>3491</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>61093</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>100978</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>43562</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>70311</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>34183</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>55791</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>39339</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>81495</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>38663</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>45296</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>18910</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>24353</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>21779</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>81771</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>65715</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>115622</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>62248</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>30477</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>61234</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>129272</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>131994</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>16241</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>95839</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>4219</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>83269</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>2725</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>55299</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>76089</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>110971</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>114992</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>73663</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>88193</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>11162</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>103966</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>125221</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>46088</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>49208</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>48021</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>111579</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>40576</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>28693</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>96872</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>116943</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>78020</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>49983</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>35597</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>98109</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>103983</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>104575</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>18340</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>30696</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>13765</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>78196</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>64376</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>59309</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>74512</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>107423</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>72190</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>71256</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>39650</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>119471</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>80325</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>26414</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>30301</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>10122</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>